<commit_message>
Set column widths on Sheet2 of the common-tables list
Only the widths of columns A, B, F and G on Sheet2 changed; no cell content was changed.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/resources/List of common tables with arch objects and clean up.xlsx
+++ b/backend/resources/List of common tables with arch objects and clean up.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sandrao7\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amedeloitte-my.sharepoint.com/personal/ritwichatterjee_deloitte_com/Documents/Desktop/SAP Assessment Automation/backend/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{912D1DDF-17C6-4EA3-9CCB-58D43E28C1F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{912D1DDF-17C6-4EA3-9CCB-58D43E28C1F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE584A75-44F8-4276-B466-36307195BD6C}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{E891F7C5-17C3-4337-9CAC-B7F9D15CF5BD}"/>
   </bookViews>
@@ -749,12 +749,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1131,1138 +1130,1138 @@
   <dimension ref="A1:F69"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.81640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="51.26953125" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.81640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.81640625" style="7" customWidth="1"/>
-    <col min="5" max="5" width="34.36328125" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="147.26953125" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.7265625" style="7"/>
+    <col min="1" max="1" width="21.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.26953125" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.81640625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="34.36328125" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="147.26953125" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.7265625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="E2" s="6"/>
-      <c r="F2" s="16"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="15"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="E3" s="8"/>
-      <c r="F3" s="16"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="15"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="E4" s="8"/>
-      <c r="F4" s="16"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="15"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="E5" s="6"/>
-      <c r="F5" s="16"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="15"/>
     </row>
     <row r="6" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="E6" s="9"/>
-      <c r="F6" s="16"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="15"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="E7" s="6"/>
-      <c r="F7" s="16"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="15"/>
     </row>
     <row r="8" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="E8" s="9"/>
-      <c r="F8" s="16"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="15"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="15" t="s">
         <v>154</v>
       </c>
-      <c r="E9" s="9"/>
-      <c r="F9" s="16"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="15"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="D10" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="E10" s="9"/>
-      <c r="F10" s="16"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="15"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="15" t="s">
         <v>172</v>
       </c>
-      <c r="E11" s="9"/>
-      <c r="F11" s="16"/>
-    </row>
-    <row r="12" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="16" t="s">
+      <c r="E11" s="8"/>
+      <c r="F11" s="15"/>
+    </row>
+    <row r="12" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="15" t="s">
         <v>154</v>
       </c>
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="15" t="s">
         <v>175</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="D12" s="16" t="s">
+      <c r="D12" s="15" t="s">
         <v>154</v>
       </c>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-    </row>
-    <row r="13" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="16" t="s">
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+    </row>
+    <row r="13" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-    </row>
-    <row r="14" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="16" t="s">
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+    </row>
+    <row r="14" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="15" t="s">
         <v>172</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="15" t="s">
         <v>180</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="D14" s="16" t="s">
+      <c r="D14" s="15" t="s">
         <v>172</v>
       </c>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="E15" s="6"/>
-      <c r="F15" s="16"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="15"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="E16" s="6"/>
-      <c r="F16" s="16"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="15"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6" t="s">
+      <c r="E17" s="5"/>
+      <c r="F17" s="5" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D20" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E20" s="6"/>
-      <c r="F20" s="16"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="15"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D21" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="E21" s="6"/>
-      <c r="F21" s="16"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="15"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D22" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="E22" s="6"/>
-      <c r="F22" s="16"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="15"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6" t="s">
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="58" x14ac:dyDescent="0.35">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6" t="s">
+      <c r="B24" s="5"/>
+      <c r="C24" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="8" t="s">
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="7" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="6" t="s">
+      <c r="A25" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="D25" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="E25" s="6"/>
-      <c r="F25" s="16" t="s">
+      <c r="E25" s="5"/>
+      <c r="F25" s="15" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A26" s="11" t="s">
+      <c r="A26" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="D26" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="E26" s="6"/>
-      <c r="F26" s="16"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="15"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="D27" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="E27" s="6"/>
-      <c r="F27" s="16"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="15"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A28" s="6" t="s">
+      <c r="A28" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D28" s="6" t="s">
+      <c r="D28" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="E28" s="6"/>
-      <c r="F28" s="16"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="15"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A29" s="6" t="s">
+      <c r="A29" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D29" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="E29" s="6"/>
-      <c r="F29" s="16"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="15"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="D30" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="E30" s="6"/>
-      <c r="F30" s="16"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="15"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A31" s="6" t="s">
+      <c r="A31" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="D31" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="E31" s="6"/>
-      <c r="F31" s="16"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="15"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A32" s="6" t="s">
+      <c r="A32" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C32" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D32" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="E32" s="6"/>
-      <c r="F32" s="16"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="15"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A33" s="6" t="s">
+      <c r="A33" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C33" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="D33" s="6"/>
-      <c r="E33" s="6"/>
-      <c r="F33" s="16"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="15"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A34" s="6" t="s">
+      <c r="A34" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="C34" s="6" t="s">
+      <c r="C34" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="D34" s="6" t="s">
+      <c r="D34" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="E34" s="6"/>
-      <c r="F34" s="16"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="15"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A35" s="6" t="s">
+      <c r="A35" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="C35" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="D35" s="9" t="s">
+      <c r="D35" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="E35" s="9"/>
-      <c r="F35" s="16"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="15"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A36" s="16" t="s">
+      <c r="A36" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="B36" s="16" t="s">
+      <c r="B36" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="C36" s="16" t="s">
+      <c r="C36" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="D36" s="16" t="s">
+      <c r="D36" s="15" t="s">
         <v>170</v>
       </c>
-      <c r="E36" s="16"/>
-      <c r="F36" s="16"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A37" s="16" t="s">
+      <c r="A37" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="B37" s="16" t="s">
+      <c r="B37" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C37" s="16" t="s">
+      <c r="C37" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="D37" s="16" t="s">
+      <c r="D37" s="15" t="s">
         <v>170</v>
       </c>
-      <c r="E37" s="16"/>
-      <c r="F37" s="16"/>
+      <c r="E37" s="15"/>
+      <c r="F37" s="15"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A38" s="16" t="s">
+      <c r="A38" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="B38" s="16" t="s">
+      <c r="B38" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="C38" s="16" t="s">
+      <c r="C38" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="D38" s="16" t="s">
+      <c r="D38" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="E38" s="16"/>
-      <c r="F38" s="16"/>
+      <c r="E38" s="15"/>
+      <c r="F38" s="15"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A39" s="16" t="s">
+      <c r="A39" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="B39" s="16" t="s">
+      <c r="B39" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="C39" s="16" t="s">
+      <c r="C39" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="D39" s="16" t="s">
+      <c r="D39" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="E39" s="16"/>
-      <c r="F39" s="16"/>
+      <c r="E39" s="15"/>
+      <c r="F39" s="15"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A40" s="16" t="s">
+      <c r="A40" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="B40" s="16" t="s">
+      <c r="B40" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="C40" s="16" t="s">
+      <c r="C40" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="D40" s="16" t="s">
+      <c r="D40" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="E40" s="16"/>
-      <c r="F40" s="16"/>
+      <c r="E40" s="15"/>
+      <c r="F40" s="15"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A41" s="16" t="s">
+      <c r="A41" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="B41" s="16" t="s">
+      <c r="B41" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="C41" s="16" t="s">
+      <c r="C41" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="D41" s="16" t="s">
+      <c r="D41" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="E41" s="16"/>
-      <c r="F41" s="16"/>
+      <c r="E41" s="15"/>
+      <c r="F41" s="15"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A42" s="16" t="s">
+      <c r="A42" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="B42" s="16" t="s">
+      <c r="B42" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="C42" s="12" t="s">
+      <c r="C42" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D42" s="12" t="s">
+      <c r="D42" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="E42" s="16"/>
-      <c r="F42" s="16"/>
+      <c r="E42" s="15"/>
+      <c r="F42" s="15"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A43" s="16" t="s">
+      <c r="A43" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="B43" s="16" t="s">
+      <c r="B43" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="C43" s="12" t="s">
+      <c r="C43" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="D43" s="12" t="s">
+      <c r="D43" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="E43" s="16"/>
-      <c r="F43" s="16"/>
+      <c r="E43" s="15"/>
+      <c r="F43" s="15"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A44" s="12" t="s">
+      <c r="A44" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="B44" s="6" t="s">
+      <c r="B44" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="C44" s="16" t="s">
+      <c r="C44" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="D44" s="16" t="s">
+      <c r="D44" s="15" t="s">
         <v>139</v>
       </c>
-      <c r="E44" s="16"/>
-      <c r="F44" s="16"/>
+      <c r="E44" s="15"/>
+      <c r="F44" s="15"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A45" s="16" t="s">
+      <c r="A45" s="15" t="s">
         <v>140</v>
       </c>
-      <c r="B45" s="16" t="s">
+      <c r="B45" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="C45" s="16" t="s">
+      <c r="C45" s="15" t="s">
         <v>144</v>
       </c>
-      <c r="D45" s="16" t="s">
+      <c r="D45" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="E45" s="16"/>
-      <c r="F45" s="16"/>
+      <c r="E45" s="15"/>
+      <c r="F45" s="15"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A46" s="16" t="s">
+      <c r="A46" s="15" t="s">
         <v>142</v>
       </c>
-      <c r="B46" s="16" t="s">
+      <c r="B46" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="C46" s="16" t="s">
+      <c r="C46" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="D46" s="16" t="s">
+      <c r="D46" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="E46" s="16"/>
-      <c r="F46" s="16"/>
+      <c r="E46" s="15"/>
+      <c r="F46" s="15"/>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A47" s="6" t="s">
+      <c r="A47" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="B47" s="6" t="s">
+      <c r="B47" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="C47" s="16" t="s">
+      <c r="C47" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="D47" s="16" t="s">
+      <c r="D47" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="E47" s="16"/>
-      <c r="F47" s="16"/>
+      <c r="E47" s="15"/>
+      <c r="F47" s="15"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A48" s="6" t="s">
+      <c r="A48" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="B48" s="6" t="s">
+      <c r="B48" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="C48" s="16" t="s">
+      <c r="C48" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="D48" s="16" t="s">
+      <c r="D48" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="E48" s="16"/>
-      <c r="F48" s="16"/>
+      <c r="E48" s="15"/>
+      <c r="F48" s="15"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A49" s="6" t="s">
+      <c r="A49" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="B49" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C49" s="16" t="s">
+      <c r="C49" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D49" s="16"/>
-      <c r="E49" s="16"/>
-      <c r="F49" s="6" t="s">
+      <c r="D49" s="15"/>
+      <c r="E49" s="15"/>
+      <c r="F49" s="5" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A50" s="6" t="s">
+      <c r="A50" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="B50" s="16" t="s">
+      <c r="B50" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="C50" s="16" t="s">
+      <c r="C50" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D50" s="16"/>
-      <c r="E50" s="16"/>
-      <c r="F50" s="6" t="s">
+      <c r="D50" s="15"/>
+      <c r="E50" s="15"/>
+      <c r="F50" s="5" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A51" s="16" t="s">
+      <c r="A51" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="B51" s="16" t="s">
+      <c r="B51" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="C51" s="16" t="s">
+      <c r="C51" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D51" s="16"/>
-      <c r="E51" s="16" t="s">
+      <c r="D51" s="15"/>
+      <c r="E51" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="F51" s="16" t="s">
+      <c r="F51" s="15" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A52" s="6" t="s">
+      <c r="A52" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B52" s="6" t="s">
+      <c r="B52" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C52" s="6" t="s">
+      <c r="C52" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D52" s="6"/>
-      <c r="E52" s="6"/>
-      <c r="F52" s="6" t="s">
+      <c r="D52" s="5"/>
+      <c r="E52" s="5"/>
+      <c r="F52" s="5" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="A53" s="6" t="s">
+      <c r="A53" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="B53" s="6" t="s">
+      <c r="B53" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="C53" s="16" t="s">
+      <c r="C53" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D53" s="16"/>
-      <c r="E53" s="16" t="s">
+      <c r="D53" s="15"/>
+      <c r="E53" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="F53" s="8" t="s">
+      <c r="F53" s="7" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A54" s="16" t="s">
+      <c r="A54" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="B54" s="16" t="s">
+      <c r="B54" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="C54" s="16" t="s">
+      <c r="C54" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D54" s="16"/>
-      <c r="E54" s="16" t="s">
+      <c r="D54" s="15"/>
+      <c r="E54" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="F54" s="8" t="s">
+      <c r="F54" s="7" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A55" s="16" t="s">
+      <c r="A55" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="B55" s="16" t="s">
+      <c r="B55" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="C55" s="16" t="s">
+      <c r="C55" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D55" s="16"/>
-      <c r="E55" s="16" t="s">
+      <c r="D55" s="15"/>
+      <c r="E55" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="F55" s="16"/>
+      <c r="F55" s="15"/>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A56" s="16" t="s">
+      <c r="A56" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="B56" s="16" t="s">
+      <c r="B56" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="C56" s="16" t="s">
+      <c r="C56" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D56" s="16"/>
-      <c r="E56" s="16" t="s">
+      <c r="D56" s="15"/>
+      <c r="E56" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="F56" s="16"/>
+      <c r="F56" s="15"/>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A57" s="16" t="s">
+      <c r="A57" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="B57" s="16" t="s">
+      <c r="B57" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="C57" s="16" t="s">
+      <c r="C57" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D57" s="16"/>
-      <c r="E57" s="16" t="s">
+      <c r="D57" s="15"/>
+      <c r="E57" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="F57" s="16"/>
+      <c r="F57" s="15"/>
     </row>
     <row r="58" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A58" s="16" t="s">
+      <c r="A58" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="B58" s="16" t="s">
+      <c r="B58" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="C58" s="16" t="s">
+      <c r="C58" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D58" s="16"/>
-      <c r="E58" s="16" t="s">
+      <c r="D58" s="15"/>
+      <c r="E58" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="F58" s="16" t="s">
+      <c r="F58" s="15" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A59" s="16" t="s">
+      <c r="A59" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="B59" s="16" t="s">
+      <c r="B59" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="C59" s="16" t="s">
+      <c r="C59" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D59" s="16"/>
-      <c r="E59" s="16" t="s">
+      <c r="D59" s="15"/>
+      <c r="E59" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="F59" s="16" t="s">
+      <c r="F59" s="15" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="60" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A60" s="16" t="s">
+      <c r="A60" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="B60" s="16" t="s">
+      <c r="B60" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="C60" s="16" t="s">
+      <c r="C60" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D60" s="16"/>
-      <c r="E60" s="16" t="s">
+      <c r="D60" s="15"/>
+      <c r="E60" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="F60" s="8" t="s">
+      <c r="F60" s="7" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A61" s="16" t="s">
+      <c r="A61" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="B61" s="16" t="s">
+      <c r="B61" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="C61" s="16" t="s">
+      <c r="C61" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D61" s="16"/>
-      <c r="E61" s="16" t="s">
+      <c r="D61" s="15"/>
+      <c r="E61" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="F61" s="16" t="s">
+      <c r="F61" s="15" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A62" s="16" t="s">
+      <c r="A62" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="B62" s="16" t="s">
+      <c r="B62" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="C62" s="16" t="s">
+      <c r="C62" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D62" s="16"/>
-      <c r="E62" s="16" t="s">
+      <c r="D62" s="15"/>
+      <c r="E62" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="F62" s="16" t="s">
+      <c r="F62" s="15" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A63" s="16" t="s">
+      <c r="A63" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="B63" s="16" t="s">
+      <c r="B63" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="C63" s="16" t="s">
+      <c r="C63" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D63" s="16"/>
-      <c r="E63" s="16" t="s">
+      <c r="D63" s="15"/>
+      <c r="E63" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="F63" s="16"/>
+      <c r="F63" s="15"/>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A64" s="14" t="s">
+      <c r="A64" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="B64" s="14" t="s">
+      <c r="B64" s="13" t="s">
         <v>187</v>
       </c>
-      <c r="C64" s="16" t="s">
+      <c r="C64" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D64" s="13"/>
-      <c r="E64" s="14" t="s">
+      <c r="D64" s="12"/>
+      <c r="E64" s="13" t="s">
         <v>192</v>
       </c>
-      <c r="F64" s="13"/>
+      <c r="F64" s="12"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A65" s="14" t="s">
+      <c r="A65" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="B65" s="14" t="s">
+      <c r="B65" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="C65" s="16" t="s">
+      <c r="C65" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D65" s="13"/>
-      <c r="E65" s="14" t="s">
+      <c r="D65" s="12"/>
+      <c r="E65" s="13" t="s">
         <v>192</v>
       </c>
-      <c r="F65" s="13"/>
+      <c r="F65" s="12"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A66" s="14" t="s">
+      <c r="A66" s="13" t="s">
         <v>184</v>
       </c>
-      <c r="B66" s="14" t="s">
+      <c r="B66" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="C66" s="16" t="s">
+      <c r="C66" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D66" s="13"/>
-      <c r="E66" s="14" t="s">
+      <c r="D66" s="12"/>
+      <c r="E66" s="13" t="s">
         <v>192</v>
       </c>
-      <c r="F66" s="13"/>
+      <c r="F66" s="12"/>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A67" s="14" t="s">
+      <c r="A67" s="13" t="s">
         <v>190</v>
       </c>
-      <c r="B67" s="14" t="s">
+      <c r="B67" s="13" t="s">
         <v>191</v>
       </c>
-      <c r="C67" s="16" t="s">
+      <c r="C67" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D67" s="13"/>
-      <c r="E67" s="14" t="s">
+      <c r="D67" s="12"/>
+      <c r="E67" s="13" t="s">
         <v>192</v>
       </c>
-      <c r="F67" s="13"/>
+      <c r="F67" s="12"/>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A68" s="14" t="s">
+      <c r="A68" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="B68" s="14" t="s">
+      <c r="B68" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="C68" s="16" t="s">
+      <c r="C68" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D68" s="13"/>
-      <c r="E68" s="14" t="s">
+      <c r="D68" s="12"/>
+      <c r="E68" s="13" t="s">
         <v>193</v>
       </c>
-      <c r="F68" s="15" t="s">
+      <c r="F68" s="14" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A69" s="14" t="s">
+      <c r="A69" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="B69" s="14" t="s">
+      <c r="B69" s="13" t="s">
         <v>196</v>
       </c>
-      <c r="C69" s="16"/>
-      <c r="D69" s="14"/>
-      <c r="E69" s="14" t="s">
+      <c r="C69" s="15"/>
+      <c r="D69" s="13"/>
+      <c r="E69" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="F69" s="13"/>
+      <c r="F69" s="12"/>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
@@ -2277,162 +2276,117 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{181CBA54-0784-4F79-969D-5806C6822741}">
   <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="34.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.1796875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+      <c r="A1" t="s">
         <v>81</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>82</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2" t="s">
+      <c r="F1" t="s">
         <v>83</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="232" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" t="s">
         <v>85</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>86</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2" t="s">
+      <c r="F2" t="s">
         <v>87</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="409.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="A3" t="s">
         <v>89</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" t="s">
         <v>90</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2" t="s">
+      <c r="F3" t="s">
         <v>91</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="2" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="A4" t="s">
         <v>93</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" t="s">
         <v>94</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2" t="s">
+      <c r="F4" t="s">
         <v>95</v>
       </c>
-      <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="A5" t="s">
         <v>96</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" t="s">
         <v>97</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2" t="s">
+      <c r="F5" t="s">
         <v>98</v>
       </c>
-      <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+      <c r="A6" t="s">
         <v>99</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" t="s">
         <v>100</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2" t="s">
+      <c r="F6" t="s">
         <v>101</v>
       </c>
-      <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2" t="s">
+      <c r="F7" t="s">
         <v>102</v>
       </c>
-      <c r="G7" s="2"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2" t="s">
+      <c r="F8" t="s">
         <v>103</v>
       </c>
-      <c r="G8" s="2"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2" t="s">
+      <c r="F9" t="s">
         <v>104</v>
       </c>
-      <c r="G9" s="2"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2" t="s">
+      <c r="F10" t="s">
         <v>105</v>
       </c>
-      <c r="G10" s="2"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2" t="s">
+      <c r="F11" t="s">
         <v>106</v>
       </c>
-      <c r="G11" s="2"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2" t="s">
+      <c r="F12" t="s">
         <v>107</v>
       </c>
-      <c r="G12" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>